<commit_message>
CD-226: Validate user inputted data file checksums in manifests for reads
- This relates to the commit 31e2bef

- Applied the same logic to reads manifest submission as the Single-cell submission but unlike the Single-cell manifest submissions, data files have to be submitted before a reads manifest can have a successful upload

- Added tests to verify and test the logic

- All unit tests and Playwright tests except for the unit test, `test_clean_str_removes_zero_width_space`, which is expected to fail

- The test manifest, `copo_single_cell_manifest_version_faang_sc_rnaseq_success1.xlsx`, was updated with correct and valid checksums matching the data files inputted in it. The checksums in the `File md5 checksum` column in `expression_data_file` worksheet as well as in the `Read 1 Checksum` column and `Read 2 Checksum` column in the `file` worksheet were updated.
</commit_message>
<xml_diff>
--- a/test/testfiles/copo_single_cell_manifest_version_faang_sc_rnaseq_success1.xlsx
+++ b/test/testfiles/copo_single_cell_manifest_version_faang_sc_rnaseq_success1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/providen/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/providen/Documents/EI/Projects/COPO-production/test/testfiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22692190-7F91-0341-BE94-E9EF55F289CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC9A92C4-3CF3-AB4A-B99C-CB24D467B468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="660" windowWidth="25360" windowHeight="12900" firstSheet="9" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="70060" yWindow="2560" windowWidth="36240" windowHeight="12900" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="study" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="601">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="602">
   <si>
     <t>Study ID</t>
   </si>
@@ -1815,9 +1815,6 @@
     <t>single_cell_index1_4.fastq.gz</t>
   </si>
   <si>
-    <t>61df53f6dc6a88b8c564378365e354f8</t>
-  </si>
-  <si>
     <t>single_cell_index2_4.fastq.gz</t>
   </si>
   <si>
@@ -1852,6 +1849,12 @@
   </si>
   <si>
     <t>h5ad</t>
+  </si>
+  <si>
+    <t>3181f0f98825ca11a47185e9d534a2b7</t>
+  </si>
+  <si>
+    <t>eb3baea9e6df8b033dbe0495765286ce</t>
   </si>
 </sst>
 </file>
@@ -8086,22 +8089,22 @@
         <v>586</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>587</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>588</v>
+        <v>600</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>515</v>
+        <v>600</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="6" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -9994,16 +9997,16 @@
         <v>530</v>
       </c>
       <c r="F5" s="3" t="s">
+        <v>591</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>592</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>593</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>539</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="K5" s="3">
         <v>1.9</v>
@@ -10012,16 +10015,16 @@
         <v>549</v>
       </c>
       <c r="M5" s="3" t="s">
+        <v>594</v>
+      </c>
+      <c r="N5" s="3" t="s">
         <v>595</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="O5" s="3" t="s">
         <v>596</v>
       </c>
-      <c r="O5" s="3" t="s">
+      <c r="P5" s="3" t="s">
         <v>597</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="6" spans="1:16" s="3" customFormat="1" x14ac:dyDescent="0.2">
@@ -11874,13 +11877,13 @@
         <v>521</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>598</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>601</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>599</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>566</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>600</v>
       </c>
       <c r="H5" s="3">
         <v>4</v>

</xml_diff>